<commit_message>
the code now works again but with the new datasheet added to it.
</commit_message>
<xml_diff>
--- a/data/Datasheet PSE 2026.xlsx
+++ b/data/Datasheet PSE 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jobna\Desktop\UNI_Git_Projecten\ProjectModule11\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3593BCAE-5271-4407-A21C-1841F11037D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3A95EE-C8B2-4AD7-BC7C-E7927808CAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" tabRatio="769" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="769" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product portfolio" sheetId="11" r:id="rId1"/>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="183">
   <si>
     <t>A</t>
   </si>
@@ -855,6 +855,30 @@
   <si>
     <t xml:space="preserve">Price per part (€) </t>
   </si>
+  <si>
+    <t>AGR-053-01</t>
+  </si>
+  <si>
+    <t>AGR-053-02</t>
+  </si>
+  <si>
+    <t>AGR-053-03</t>
+  </si>
+  <si>
+    <t>AGR-053-04</t>
+  </si>
+  <si>
+    <t>AGR-053-05</t>
+  </si>
+  <si>
+    <t>AGR-053-06</t>
+  </si>
+  <si>
+    <t>AGR-053-07</t>
+  </si>
+  <si>
+    <t>AGR-053-08</t>
+  </si>
 </sst>
 </file>
 
@@ -865,7 +889,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -938,6 +962,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -976,7 +1006,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1049,6 +1079,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1336,7 +1374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P287"/>
+  <dimension ref="A1:P330"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -7759,6 +7797,1031 @@
       <c r="I287" s="2">
         <v>5.9160600070792602E-2</v>
       </c>
+    </row>
+    <row r="288" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A288" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="B288" s="34">
+        <v>10</v>
+      </c>
+      <c r="C288" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D288" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="E288" s="37">
+        <v>2</v>
+      </c>
+      <c r="F288" s="34">
+        <v>1</v>
+      </c>
+      <c r="G288" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="H288" s="35">
+        <v>2.214</v>
+      </c>
+      <c r="I288" s="35">
+        <v>0</v>
+      </c>
+      <c r="J288" s="35">
+        <v>188.54999999999998</v>
+      </c>
+      <c r="K288" s="34"/>
+    </row>
+    <row r="289" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A289" s="34"/>
+      <c r="B289" s="34"/>
+      <c r="C289" s="34"/>
+      <c r="D289" s="34" t="s">
+        <v>177</v>
+      </c>
+      <c r="E289" s="37">
+        <v>4</v>
+      </c>
+      <c r="F289" s="34"/>
+      <c r="G289" s="34"/>
+      <c r="H289" s="34"/>
+      <c r="I289" s="35"/>
+      <c r="J289" s="35"/>
+      <c r="K289" s="34"/>
+    </row>
+    <row r="290" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A290" s="34"/>
+      <c r="B290" s="34"/>
+      <c r="C290" s="34"/>
+      <c r="D290" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="E290" s="37">
+        <v>2</v>
+      </c>
+      <c r="F290" s="34"/>
+      <c r="G290" s="34"/>
+      <c r="H290" s="34"/>
+      <c r="I290" s="35"/>
+      <c r="J290" s="35"/>
+      <c r="K290" s="34"/>
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A291" s="34"/>
+      <c r="B291" s="34"/>
+      <c r="C291" s="34"/>
+      <c r="D291" s="34" t="s">
+        <v>179</v>
+      </c>
+      <c r="E291" s="37">
+        <v>1</v>
+      </c>
+      <c r="F291" s="34"/>
+      <c r="G291" s="34"/>
+      <c r="H291" s="34"/>
+      <c r="I291" s="35"/>
+      <c r="J291" s="35"/>
+      <c r="K291" s="34"/>
+    </row>
+    <row r="292" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A292" s="34"/>
+      <c r="B292" s="34"/>
+      <c r="C292" s="34"/>
+      <c r="D292" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="E292" s="37">
+        <v>3</v>
+      </c>
+      <c r="F292" s="34"/>
+      <c r="G292" s="34"/>
+      <c r="H292" s="34"/>
+      <c r="I292" s="35"/>
+      <c r="J292" s="35"/>
+      <c r="K292" s="34"/>
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A293" s="34"/>
+      <c r="B293" s="34"/>
+      <c r="C293" s="34"/>
+      <c r="D293" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="E293" s="37">
+        <v>2</v>
+      </c>
+      <c r="F293" s="34"/>
+      <c r="G293" s="34"/>
+      <c r="H293" s="34"/>
+      <c r="I293" s="35"/>
+      <c r="J293" s="35"/>
+      <c r="K293" s="34"/>
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A294" s="34"/>
+      <c r="B294" s="34"/>
+      <c r="C294" s="34"/>
+      <c r="D294" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="E294" s="37">
+        <v>4</v>
+      </c>
+      <c r="F294" s="34"/>
+      <c r="G294" s="34"/>
+      <c r="H294" s="34"/>
+      <c r="I294" s="35"/>
+      <c r="J294" s="35"/>
+      <c r="K294" s="34"/>
+    </row>
+    <row r="295" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A295" s="34"/>
+      <c r="B295" s="34"/>
+      <c r="C295" s="34"/>
+      <c r="D295" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="E295" s="37">
+        <v>3</v>
+      </c>
+      <c r="F295" s="34"/>
+      <c r="G295" s="34"/>
+      <c r="H295" s="34"/>
+      <c r="I295" s="35"/>
+      <c r="J295" s="35"/>
+      <c r="K295" s="34"/>
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A296" s="34"/>
+      <c r="B296" s="34"/>
+      <c r="C296" s="34"/>
+      <c r="D296" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="E296" s="37">
+        <v>1</v>
+      </c>
+      <c r="F296" s="34"/>
+      <c r="G296" s="34"/>
+      <c r="H296" s="34"/>
+      <c r="I296" s="35"/>
+      <c r="J296" s="35"/>
+      <c r="K296" s="34"/>
+    </row>
+    <row r="297" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A297" s="34"/>
+      <c r="B297" s="34"/>
+      <c r="C297" s="34"/>
+      <c r="D297" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="E297" s="37">
+        <v>1</v>
+      </c>
+      <c r="F297" s="34"/>
+      <c r="G297" s="34"/>
+      <c r="H297" s="34"/>
+      <c r="I297" s="35"/>
+      <c r="J297" s="35"/>
+      <c r="K297" s="34"/>
+    </row>
+    <row r="298" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A298" s="34"/>
+      <c r="B298" s="34"/>
+      <c r="C298" s="34"/>
+      <c r="D298" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="E298" s="37">
+        <v>1</v>
+      </c>
+      <c r="F298" s="34"/>
+      <c r="G298" s="34"/>
+      <c r="H298" s="34"/>
+      <c r="I298" s="35"/>
+      <c r="J298" s="35"/>
+      <c r="K298" s="34"/>
+    </row>
+    <row r="299" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A299" s="34"/>
+      <c r="B299" s="34"/>
+      <c r="C299" s="34"/>
+      <c r="D299" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="E299" s="37">
+        <v>1</v>
+      </c>
+      <c r="F299" s="34"/>
+      <c r="G299" s="34"/>
+      <c r="H299" s="34"/>
+      <c r="I299" s="35"/>
+      <c r="J299" s="35"/>
+      <c r="K299" s="34"/>
+    </row>
+    <row r="300" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A300" s="34"/>
+      <c r="B300" s="34"/>
+      <c r="C300" s="34"/>
+      <c r="D300" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E300" s="37">
+        <v>1</v>
+      </c>
+      <c r="F300" s="34"/>
+      <c r="G300" s="34"/>
+      <c r="H300" s="34"/>
+      <c r="I300" s="35"/>
+      <c r="J300" s="35"/>
+      <c r="K300" s="34"/>
+    </row>
+    <row r="301" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A301" s="34"/>
+      <c r="B301" s="34"/>
+      <c r="C301" s="34"/>
+      <c r="D301" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E301" s="37"/>
+      <c r="F301" s="34"/>
+      <c r="G301" s="34"/>
+      <c r="H301" s="34"/>
+      <c r="I301" s="35"/>
+      <c r="J301" s="35"/>
+      <c r="K301" s="34"/>
+    </row>
+    <row r="302" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A302" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="B302" s="34">
+        <v>10</v>
+      </c>
+      <c r="C302" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D302" s="34"/>
+      <c r="E302" s="34"/>
+      <c r="F302" s="34">
+        <v>20</v>
+      </c>
+      <c r="G302" s="35">
+        <v>0.7</v>
+      </c>
+      <c r="H302" s="35">
+        <v>0.49044416828866244</v>
+      </c>
+      <c r="I302" s="36">
+        <v>8.5523607660504999E-2</v>
+      </c>
+      <c r="J302" s="36">
+        <v>69.478271873497604</v>
+      </c>
+      <c r="K302" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="303" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A303" s="34"/>
+      <c r="B303" s="34">
+        <v>20</v>
+      </c>
+      <c r="C303" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="D303" s="34"/>
+      <c r="E303" s="34"/>
+      <c r="F303" s="34">
+        <v>20</v>
+      </c>
+      <c r="G303" s="35">
+        <v>1.8</v>
+      </c>
+      <c r="H303" s="35">
+        <v>0.75</v>
+      </c>
+      <c r="I303" s="36">
+        <v>9.26516014465672E-2</v>
+      </c>
+      <c r="J303" s="36"/>
+      <c r="K303" s="34"/>
+    </row>
+    <row r="304" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A304" s="34"/>
+      <c r="B304" s="34">
+        <v>30</v>
+      </c>
+      <c r="C304" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D304" s="34"/>
+      <c r="E304" s="34"/>
+      <c r="F304" s="34">
+        <v>20</v>
+      </c>
+      <c r="G304" s="35">
+        <v>0.38364285931583364</v>
+      </c>
+      <c r="H304" s="35">
+        <v>1.9039539843200504E-2</v>
+      </c>
+      <c r="I304" s="36">
+        <v>4.3344103714953598E-2</v>
+      </c>
+      <c r="J304" s="36"/>
+      <c r="K304" s="34"/>
+    </row>
+    <row r="305" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A305" s="34"/>
+      <c r="B305" s="34">
+        <v>40</v>
+      </c>
+      <c r="C305" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D305" s="34"/>
+      <c r="E305" s="34"/>
+      <c r="F305" s="34">
+        <v>20</v>
+      </c>
+      <c r="G305" s="35">
+        <v>1.192645062473638</v>
+      </c>
+      <c r="H305" s="35">
+        <v>0.19</v>
+      </c>
+      <c r="I305" s="36">
+        <v>5.9160600070792602E-2</v>
+      </c>
+      <c r="J305" s="36"/>
+      <c r="K305" s="34"/>
+    </row>
+    <row r="306" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A306" s="34"/>
+      <c r="B306" s="34">
+        <v>50</v>
+      </c>
+      <c r="C306" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D306" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E306" s="34"/>
+      <c r="F306" s="34">
+        <v>40</v>
+      </c>
+      <c r="G306" s="35">
+        <v>3.8889304928952706E-2</v>
+      </c>
+      <c r="H306" s="35">
+        <v>0.56258096816070735</v>
+      </c>
+      <c r="I306" s="36">
+        <v>0.134941999254343</v>
+      </c>
+      <c r="J306" s="36"/>
+      <c r="K306" s="34"/>
+    </row>
+    <row r="307" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A307" s="34" t="s">
+        <v>177</v>
+      </c>
+      <c r="B307" s="34">
+        <v>10</v>
+      </c>
+      <c r="C307" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D307" s="34"/>
+      <c r="E307" s="34"/>
+      <c r="F307" s="34">
+        <v>40</v>
+      </c>
+      <c r="G307" s="35">
+        <v>1.5320301793168802</v>
+      </c>
+      <c r="H307" s="35">
+        <v>0.24080177919334866</v>
+      </c>
+      <c r="I307" s="36">
+        <v>8.5523607660504999E-2</v>
+      </c>
+      <c r="J307" s="36">
+        <v>42.585735309263086</v>
+      </c>
+      <c r="K307" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="308" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A308" s="34"/>
+      <c r="B308" s="34">
+        <v>20</v>
+      </c>
+      <c r="C308" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D308" s="34"/>
+      <c r="E308" s="34"/>
+      <c r="F308" s="34">
+        <v>40</v>
+      </c>
+      <c r="G308" s="35">
+        <v>0.94036017650040415</v>
+      </c>
+      <c r="H308" s="35">
+        <v>0.1419947423658805</v>
+      </c>
+      <c r="I308" s="36">
+        <v>5.0533608893815203E-2</v>
+      </c>
+      <c r="J308" s="36"/>
+      <c r="K308" s="34"/>
+    </row>
+    <row r="309" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A309" s="34"/>
+      <c r="B309" s="34">
+        <v>30</v>
+      </c>
+      <c r="C309" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D309" s="34"/>
+      <c r="E309" s="34"/>
+      <c r="F309" s="34">
+        <v>40</v>
+      </c>
+      <c r="G309" s="35">
+        <v>1.7925361354309186</v>
+      </c>
+      <c r="H309" s="35">
+        <v>0.17086296361734199</v>
+      </c>
+      <c r="I309" s="36">
+        <v>3.50421596453767E-2</v>
+      </c>
+      <c r="J309" s="36"/>
+      <c r="K309" s="34"/>
+    </row>
+    <row r="310" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A310" s="34"/>
+      <c r="B310" s="34">
+        <v>40</v>
+      </c>
+      <c r="C310" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D310" s="34"/>
+      <c r="E310" s="34"/>
+      <c r="F310" s="34">
+        <v>40</v>
+      </c>
+      <c r="G310" s="35">
+        <v>1.1767819642559467</v>
+      </c>
+      <c r="H310" s="35">
+        <v>0.23</v>
+      </c>
+      <c r="I310" s="36">
+        <v>5.9160600070792602E-2</v>
+      </c>
+      <c r="J310" s="36"/>
+      <c r="K310" s="34"/>
+    </row>
+    <row r="311" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A311" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="B311" s="34">
+        <v>10</v>
+      </c>
+      <c r="C311" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D311" s="34"/>
+      <c r="E311" s="34"/>
+      <c r="F311" s="34">
+        <v>20</v>
+      </c>
+      <c r="G311" s="35">
+        <v>0.9452997296870298</v>
+      </c>
+      <c r="H311" s="35">
+        <v>0.46869742578798812</v>
+      </c>
+      <c r="I311" s="36">
+        <v>8.5523607660504999E-2</v>
+      </c>
+      <c r="J311" s="36">
+        <v>57.676389304676952</v>
+      </c>
+      <c r="K311" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="312" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A312" s="34"/>
+      <c r="B312" s="34">
+        <v>20</v>
+      </c>
+      <c r="C312" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="D312" s="34"/>
+      <c r="E312" s="34"/>
+      <c r="F312" s="34">
+        <v>20</v>
+      </c>
+      <c r="G312" s="35">
+        <v>2.1</v>
+      </c>
+      <c r="H312" s="35">
+        <v>0.21954512416657479</v>
+      </c>
+      <c r="I312" s="36">
+        <v>9.26516014465672E-2</v>
+      </c>
+      <c r="J312" s="36"/>
+      <c r="K312" s="34"/>
+    </row>
+    <row r="313" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A313" s="34"/>
+      <c r="B313" s="34">
+        <v>30</v>
+      </c>
+      <c r="C313" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D313" s="34"/>
+      <c r="E313" s="34"/>
+      <c r="F313" s="34">
+        <v>20</v>
+      </c>
+      <c r="G313" s="35">
+        <v>1.2844228509279483</v>
+      </c>
+      <c r="H313" s="35">
+        <v>0.67457253901450709</v>
+      </c>
+      <c r="I313" s="36">
+        <v>4.3344103714953598E-2</v>
+      </c>
+      <c r="J313" s="36"/>
+      <c r="K313" s="34"/>
+    </row>
+    <row r="314" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A314" s="34"/>
+      <c r="B314" s="34">
+        <v>40</v>
+      </c>
+      <c r="C314" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D314" s="34"/>
+      <c r="E314" s="34"/>
+      <c r="F314" s="34">
+        <v>20</v>
+      </c>
+      <c r="G314" s="35">
+        <v>1.8523663879175478</v>
+      </c>
+      <c r="H314" s="35">
+        <v>0.15183635308622023</v>
+      </c>
+      <c r="I314" s="36">
+        <v>5.9160600070792602E-2</v>
+      </c>
+      <c r="J314" s="36"/>
+      <c r="K314" s="34"/>
+    </row>
+    <row r="315" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A315" s="34"/>
+      <c r="B315" s="34">
+        <v>50</v>
+      </c>
+      <c r="C315" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D315" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E315" s="34"/>
+      <c r="F315" s="34">
+        <v>40</v>
+      </c>
+      <c r="G315" s="35">
+        <v>0.4</v>
+      </c>
+      <c r="H315" s="35">
+        <v>0.27625308872995746</v>
+      </c>
+      <c r="I315" s="36">
+        <v>0.134941999254343</v>
+      </c>
+      <c r="J315" s="36"/>
+      <c r="K315" s="34"/>
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A316" s="34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B316" s="34">
+        <v>10</v>
+      </c>
+      <c r="C316" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D316" s="34"/>
+      <c r="E316" s="34"/>
+      <c r="F316" s="34">
+        <v>20</v>
+      </c>
+      <c r="G316" s="35">
+        <v>0.16910372521292483</v>
+      </c>
+      <c r="H316" s="35">
+        <v>0.62390114044437051</v>
+      </c>
+      <c r="I316" s="36">
+        <v>8.5523607660504999E-2</v>
+      </c>
+      <c r="J316" s="36">
+        <v>379.75930221539681</v>
+      </c>
+      <c r="K316" s="34" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="317" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A317" s="34"/>
+      <c r="B317" s="34">
+        <v>20</v>
+      </c>
+      <c r="C317" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="D317" s="34"/>
+      <c r="E317" s="34"/>
+      <c r="F317" s="34">
+        <v>20</v>
+      </c>
+      <c r="G317" s="35">
+        <v>0.66093568275210823</v>
+      </c>
+      <c r="H317" s="35">
+        <v>0.80672818589092732</v>
+      </c>
+      <c r="I317" s="36">
+        <v>0.111421850244242</v>
+      </c>
+      <c r="J317" s="36"/>
+      <c r="K317" s="34"/>
+    </row>
+    <row r="318" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A318" s="34"/>
+      <c r="B318" s="34">
+        <v>30</v>
+      </c>
+      <c r="C318" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D318" s="34"/>
+      <c r="E318" s="34"/>
+      <c r="F318" s="34">
+        <v>20</v>
+      </c>
+      <c r="G318" s="35">
+        <v>1.9542262227447631</v>
+      </c>
+      <c r="H318" s="35">
+        <v>0.88687904122446926</v>
+      </c>
+      <c r="I318" s="36">
+        <v>5.0533608893815203E-2</v>
+      </c>
+      <c r="J318" s="36"/>
+      <c r="K318" s="34"/>
+    </row>
+    <row r="319" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A319" s="34"/>
+      <c r="B319" s="34">
+        <v>40</v>
+      </c>
+      <c r="C319" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D319" s="34"/>
+      <c r="E319" s="34"/>
+      <c r="F319" s="34">
+        <v>20</v>
+      </c>
+      <c r="G319" s="35">
+        <v>0.97895493951619605</v>
+      </c>
+      <c r="H319" s="35">
+        <v>0.82285041506711221</v>
+      </c>
+      <c r="I319" s="36">
+        <v>4.3344103714953598E-2</v>
+      </c>
+      <c r="J319" s="36"/>
+      <c r="K319" s="34"/>
+    </row>
+    <row r="320" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A320" s="34"/>
+      <c r="B320" s="34">
+        <v>50</v>
+      </c>
+      <c r="C320" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D320" s="34"/>
+      <c r="E320" s="34"/>
+      <c r="F320" s="34">
+        <v>20</v>
+      </c>
+      <c r="G320" s="35">
+        <v>0.7916615927779751</v>
+      </c>
+      <c r="H320" s="35">
+        <v>0.24</v>
+      </c>
+      <c r="I320" s="36">
+        <v>5.9160600070792602E-2</v>
+      </c>
+      <c r="J320" s="36"/>
+      <c r="K320" s="34"/>
+    </row>
+    <row r="321" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A321" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="B321" s="34">
+        <v>10</v>
+      </c>
+      <c r="C321" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D321" s="34"/>
+      <c r="E321" s="34"/>
+      <c r="F321" s="34">
+        <v>20</v>
+      </c>
+      <c r="G321" s="35">
+        <v>0</v>
+      </c>
+      <c r="H321" s="35">
+        <v>0.41599979921119845</v>
+      </c>
+      <c r="I321" s="36">
+        <v>8.5523607660504999E-2</v>
+      </c>
+      <c r="J321" s="36">
+        <v>61.714603314224242</v>
+      </c>
+      <c r="K321" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="322" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A322" s="34"/>
+      <c r="B322" s="34">
+        <v>20</v>
+      </c>
+      <c r="C322" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="D322" s="34"/>
+      <c r="E322" s="34"/>
+      <c r="F322" s="34">
+        <v>20</v>
+      </c>
+      <c r="G322" s="35">
+        <v>1.1264938856419069</v>
+      </c>
+      <c r="H322" s="35">
+        <v>0.12894269349985998</v>
+      </c>
+      <c r="I322" s="36">
+        <v>0.111421850244242</v>
+      </c>
+      <c r="J322" s="36"/>
+      <c r="K322" s="34"/>
+    </row>
+    <row r="323" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A323" s="34"/>
+      <c r="B323" s="34">
+        <v>30</v>
+      </c>
+      <c r="C323" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D323" s="34"/>
+      <c r="E323" s="34"/>
+      <c r="F323" s="34">
+        <v>20</v>
+      </c>
+      <c r="G323" s="35">
+        <v>0.47589854172011603</v>
+      </c>
+      <c r="H323" s="35">
+        <v>0.50133709796108217</v>
+      </c>
+      <c r="I323" s="36">
+        <v>5.0533608893815203E-2</v>
+      </c>
+      <c r="J323" s="36"/>
+      <c r="K323" s="34"/>
+    </row>
+    <row r="324" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A324" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="B324" s="34">
+        <v>10</v>
+      </c>
+      <c r="C324" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="D324" s="34"/>
+      <c r="E324" s="34"/>
+      <c r="F324" s="34">
+        <v>30</v>
+      </c>
+      <c r="G324" s="35">
+        <v>1.7</v>
+      </c>
+      <c r="H324" s="35">
+        <v>0.90987012522244037</v>
+      </c>
+      <c r="I324" s="36">
+        <v>9.26516014465672E-2</v>
+      </c>
+      <c r="J324" s="36">
+        <v>79.992923296584763</v>
+      </c>
+      <c r="K324" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="325" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A325" s="34"/>
+      <c r="B325" s="34">
+        <v>20</v>
+      </c>
+      <c r="C325" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D325" s="34"/>
+      <c r="E325" s="34"/>
+      <c r="F325" s="34">
+        <v>30</v>
+      </c>
+      <c r="G325" s="35">
+        <v>0.65249959445295591</v>
+      </c>
+      <c r="H325" s="35">
+        <v>0.22455768560596334</v>
+      </c>
+      <c r="I325" s="36">
+        <v>4.3344103714953598E-2</v>
+      </c>
+      <c r="J325" s="36"/>
+      <c r="K325" s="34"/>
+    </row>
+    <row r="326" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A326" s="34"/>
+      <c r="B326" s="34">
+        <v>30</v>
+      </c>
+      <c r="C326" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D326" s="34"/>
+      <c r="E326" s="34"/>
+      <c r="F326" s="34">
+        <v>30</v>
+      </c>
+      <c r="G326" s="35">
+        <v>0.42316334391357913</v>
+      </c>
+      <c r="H326" s="35">
+        <v>0.23</v>
+      </c>
+      <c r="I326" s="36">
+        <v>5.9160600070792602E-2</v>
+      </c>
+      <c r="J326" s="36"/>
+      <c r="K326" s="34"/>
+    </row>
+    <row r="327" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A327" s="34"/>
+      <c r="B327" s="34">
+        <v>40</v>
+      </c>
+      <c r="C327" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D327" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E327" s="34"/>
+      <c r="F327" s="34">
+        <v>30</v>
+      </c>
+      <c r="G327" s="35">
+        <v>0.69794070333499758</v>
+      </c>
+      <c r="H327" s="35">
+        <v>0.8483212410104547</v>
+      </c>
+      <c r="I327" s="36">
+        <v>0.134941999254343</v>
+      </c>
+      <c r="J327" s="36"/>
+      <c r="K327" s="34"/>
+    </row>
+    <row r="328" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A328" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="B328" s="34">
+        <v>10</v>
+      </c>
+      <c r="C328" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D328" s="34"/>
+      <c r="E328" s="34"/>
+      <c r="F328" s="34">
+        <v>30</v>
+      </c>
+      <c r="G328" s="35">
+        <v>1</v>
+      </c>
+      <c r="H328" s="35">
+        <v>1</v>
+      </c>
+      <c r="I328" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="J328" s="36">
+        <v>8.5833333333333339</v>
+      </c>
+      <c r="K328" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="329" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A329" s="34"/>
+      <c r="B329" s="34">
+        <v>20</v>
+      </c>
+      <c r="C329" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D329" s="34"/>
+      <c r="E329" s="34"/>
+      <c r="F329" s="34">
+        <v>30</v>
+      </c>
+      <c r="G329" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="H329" s="35">
+        <v>3.3</v>
+      </c>
+      <c r="I329" s="36">
+        <v>0.3</v>
+      </c>
+      <c r="J329" s="36"/>
+      <c r="K329" s="34"/>
+    </row>
+    <row r="330" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A330" s="34"/>
+      <c r="B330" s="34">
+        <v>30</v>
+      </c>
+      <c r="C330" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D330" s="34"/>
+      <c r="E330" s="34"/>
+      <c r="F330" s="34">
+        <v>30</v>
+      </c>
+      <c r="G330" s="35">
+        <v>1</v>
+      </c>
+      <c r="H330" s="35">
+        <v>2</v>
+      </c>
+      <c r="I330" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="J330" s="36"/>
+      <c r="K330" s="34"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10333,7 +11396,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{772B1D9D-C245-4E74-A616-B6AA7B075111}">
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12" style="8" bestFit="1" customWidth="1"/>
@@ -13759,7 +14822,74 @@
         <v>45987</v>
       </c>
     </row>
-    <row r="203" spans="1:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A202" s="34">
+        <v>201</v>
+      </c>
+      <c r="B202" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="C202" s="9">
+        <v>75</v>
+      </c>
+      <c r="D202" s="7">
+        <v>45870</v>
+      </c>
+      <c r="E202" s="7">
+        <v>45901</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A203" s="39">
+        <v>202</v>
+      </c>
+      <c r="B203" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="C203" s="9">
+        <v>75</v>
+      </c>
+      <c r="D203" s="7">
+        <v>45901</v>
+      </c>
+      <c r="E203" s="7">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A204" s="39">
+        <v>203</v>
+      </c>
+      <c r="B204" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="C204" s="9">
+        <v>75</v>
+      </c>
+      <c r="D204" s="7">
+        <v>45931</v>
+      </c>
+      <c r="E204" s="7">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A205" s="39">
+        <v>204</v>
+      </c>
+      <c r="B205" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="C205" s="9">
+        <v>75</v>
+      </c>
+      <c r="D205" s="7">
+        <v>45962</v>
+      </c>
+      <c r="E205" s="7">
+        <v>45992</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>